<commit_message>
Some Changes done in testng.xml
</commit_message>
<xml_diff>
--- a/autoIt/ImportFiles/BRS Import1.xlsx
+++ b/autoIt/ImportFiles/BRS Import1.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\FocusXBillWise1\BillWise\autoIt\ImportFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\FocusXBillWise1\BillWise\autoIt\ImportFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="6600" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="6600" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>

</xml_diff>